<commit_message>
Update dashboard with Myanmar language support, Material 3 Expressive styling, and petroleum transportation theme
</commit_message>
<xml_diff>
--- a/RETAIL.xlsx
+++ b/RETAIL.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ATK\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ATK\Desktop\aurum-visualization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{94A6DF1F-54A7-48CE-A303-487FA749852B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DA76FA9-2FD7-445E-A368-A9D9DAEDDAD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11310" tabRatio="745" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Apr 2025" sheetId="101" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0">'Apr 2025'!$A$1:$G$132</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Apr 2025'!$A$1:$G$132</definedName>
     <definedName name="_xlcn.WorksheetConnection_Sep2023A1AD2251" hidden="1">#REF!</definedName>
     <definedName name="Amount">#REF!</definedName>
     <definedName name="DAllo">#REF!</definedName>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="592" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="662" uniqueCount="89">
   <si>
     <t>Naing Lin Zaw</t>
   </si>
@@ -119,9 +119,6 @@
     <t>Hlaing Win</t>
   </si>
   <si>
-    <t>Win Naing (2)</t>
-  </si>
-  <si>
     <t>Khaing Min Htwe</t>
   </si>
   <si>
@@ -276,6 +273,51 @@
   </si>
   <si>
     <t>Lease</t>
+  </si>
+  <si>
+    <t>Kyaw Zin Tun</t>
+  </si>
+  <si>
+    <t>Naing Lin Aung</t>
+  </si>
+  <si>
+    <t>Moe Swe Oo</t>
+  </si>
+  <si>
+    <t>Kyaw Lin Tun</t>
+  </si>
+  <si>
+    <t>Thet Aung Tun</t>
+  </si>
+  <si>
+    <t>Pyae Sone Oo</t>
+  </si>
+  <si>
+    <t>Asaine</t>
+  </si>
+  <si>
+    <t>Paing Ye Tun</t>
+  </si>
+  <si>
+    <t>Saw Ye Naing Htwe</t>
+  </si>
+  <si>
+    <t>Saw Pawe Lah</t>
+  </si>
+  <si>
+    <t>Nyein Chan Thu</t>
+  </si>
+  <si>
+    <t>Min Ya Wai Aung</t>
+  </si>
+  <si>
+    <t>Lease Driver</t>
+  </si>
+  <si>
+    <t>Lease Helper</t>
+  </si>
+  <si>
+    <t>Win Naing</t>
   </si>
 </sst>
 </file>
@@ -819,16 +861,16 @@
   <sheetData>
     <row r="1" spans="1:7" s="15" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="16" t="s">
+        <v>70</v>
+      </c>
+      <c r="B1" s="14" t="s">
         <v>71</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="C1" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="C1" s="12" t="s">
-        <v>70</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>73</v>
       </c>
       <c r="E1" s="13" t="s">
         <v>11</v>
@@ -845,16 +887,16 @@
         <v>45748</v>
       </c>
       <c r="B2" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D2" s="3">
         <v>12723</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>17</v>
@@ -868,16 +910,16 @@
         <v>45748</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D3" s="3">
         <v>14546</v>
       </c>
       <c r="E3" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>15</v>
@@ -891,41 +933,45 @@
         <v>45748</v>
       </c>
       <c r="B4" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D4" s="3">
         <v>40000</v>
       </c>
       <c r="E4" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
+        <v>54</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="5" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8">
         <v>45748</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D5" s="3">
         <v>40000</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>22</v>
+        <v>88</v>
       </c>
       <c r="G5" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -933,10 +979,10 @@
         <v>45748</v>
       </c>
       <c r="B6" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D6" s="3">
         <v>42277</v>
@@ -945,10 +991,10 @@
         <v>5</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -956,10 +1002,10 @@
         <v>45749</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D7" s="3">
         <v>40000</v>
@@ -967,46 +1013,54 @@
       <c r="E7" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F7" s="4"/>
-      <c r="G7" s="4"/>
+      <c r="F7" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="8" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="8">
         <v>45749</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D8" s="3">
         <v>43000</v>
       </c>
       <c r="E8" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="F8" s="4"/>
-      <c r="G8" s="4"/>
+        <v>46</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G8" s="4" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="9" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="8">
         <v>45749</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D9" s="3">
         <v>40000</v>
       </c>
       <c r="E9" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G9" s="4" t="s">
         <v>18</v>
@@ -1017,16 +1071,16 @@
         <v>45749</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D10" s="3">
         <v>14546</v>
       </c>
       <c r="E10" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F10" s="4" t="s">
         <v>15</v>
@@ -1040,10 +1094,10 @@
         <v>45749</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D11" s="3">
         <v>42277</v>
@@ -1051,30 +1105,34 @@
       <c r="E11" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="F11" s="4"/>
-      <c r="G11" s="4"/>
+      <c r="F11" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="G11" s="4" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="12" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="8">
         <v>45749</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D12" s="3">
         <v>15587</v>
       </c>
       <c r="E12" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1082,29 +1140,33 @@
         <v>45749</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D13" s="3">
         <v>43000</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
+        <v>54</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="14" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="8">
         <v>45750</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D14" s="3">
         <v>42725</v>
@@ -1124,16 +1186,16 @@
         <v>45750</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D15" s="3">
         <v>12528</v>
       </c>
       <c r="E15" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F15" s="4" t="s">
         <v>17</v>
@@ -1147,22 +1209,22 @@
         <v>45750</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D16" s="3">
         <v>16365</v>
       </c>
       <c r="E16" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="17" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1170,10 +1232,10 @@
         <v>45751</v>
       </c>
       <c r="B17" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D17" s="3">
         <v>14005</v>
@@ -1193,10 +1255,10 @@
         <v>45751</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D18" s="3">
         <v>12728</v>
@@ -1216,22 +1278,22 @@
         <v>45751</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D19" s="3">
         <v>16365</v>
       </c>
       <c r="E19" s="7" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G19" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="20" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1239,10 +1301,10 @@
         <v>45751</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D20" s="3">
         <v>40000</v>
@@ -1254,7 +1316,7 @@
         <v>2</v>
       </c>
       <c r="G20" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1262,22 +1324,22 @@
         <v>45751</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D21" s="3">
         <v>40000</v>
       </c>
       <c r="E21" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F21" s="4" t="s">
         <v>19</v>
       </c>
       <c r="G21" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="22" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1285,10 +1347,10 @@
         <v>45752</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D22" s="3">
         <v>38800</v>
@@ -1296,24 +1358,28 @@
       <c r="E22" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F22" s="4"/>
-      <c r="G22" s="4"/>
+      <c r="F22" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="G22" s="4" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="23" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="8">
         <v>45752</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D23" s="3">
         <v>12728</v>
       </c>
       <c r="E23" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F23" s="4" t="s">
         <v>17</v>
@@ -1327,10 +1393,10 @@
         <v>45752</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D24" s="3">
         <v>14545</v>
@@ -1342,7 +1408,7 @@
         <v>3</v>
       </c>
       <c r="G24" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="25" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1350,10 +1416,10 @@
         <v>45753</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D25" s="3">
         <v>43000</v>
@@ -1361,37 +1427,45 @@
       <c r="E25" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F25" s="4"/>
-      <c r="G25" s="4"/>
+      <c r="F25" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G25" s="4" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="26" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="8">
         <v>45753</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D26" s="3">
         <v>43000</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="F26" s="4"/>
-      <c r="G26" s="4"/>
+        <v>46</v>
+      </c>
+      <c r="F26" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G26" s="4" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="27" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="8">
         <v>45753</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D27" s="3">
         <v>40000</v>
@@ -1400,10 +1474,10 @@
         <v>5</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1411,10 +1485,10 @@
         <v>45753</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D28" s="3">
         <v>40000</v>
@@ -1422,30 +1496,34 @@
       <c r="E28" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="F28" s="4"/>
-      <c r="G28" s="4"/>
+      <c r="F28" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="G28" s="4" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="29" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="8">
         <v>45753</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D29" s="3">
         <v>41756</v>
       </c>
       <c r="E29" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1453,22 +1531,22 @@
         <v>45753</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D30" s="3">
         <v>16355</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1476,22 +1554,22 @@
         <v>45753</v>
       </c>
       <c r="B31" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C31" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D31" s="3">
         <v>39426</v>
       </c>
       <c r="E31" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>22</v>
+        <v>88</v>
       </c>
       <c r="G31" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="32" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1499,22 +1577,22 @@
         <v>45753</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D32" s="3">
         <v>14546</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F32" s="4" t="s">
         <v>3</v>
       </c>
       <c r="G32" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="33" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1522,10 +1600,10 @@
         <v>45754</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D33" s="3">
         <v>14547</v>
@@ -1537,7 +1615,7 @@
         <v>3</v>
       </c>
       <c r="G33" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="34" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1545,16 +1623,16 @@
         <v>45754</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D34" s="3">
         <v>12265</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F34" s="4" t="s">
         <v>15</v>
@@ -1568,22 +1646,22 @@
         <v>45754</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D35" s="3">
         <v>36368</v>
       </c>
       <c r="E35" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G35" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="36" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1591,16 +1669,16 @@
         <v>45754</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D36" s="3">
         <v>42725</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F36" s="4" t="s">
         <v>21</v>
@@ -1614,10 +1692,10 @@
         <v>45755</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D37" s="3">
         <v>12728</v>
@@ -1637,22 +1715,22 @@
         <v>45755</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D38" s="3">
         <v>16365</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G38" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="39" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1660,22 +1738,22 @@
         <v>45755</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D39" s="3">
         <v>13514</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F39" s="4" t="s">
         <v>3</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="40" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1683,10 +1761,10 @@
         <v>45756</v>
       </c>
       <c r="B40" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C40" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D40" s="3">
         <v>40000</v>
@@ -1698,7 +1776,7 @@
         <v>2</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="41" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1706,10 +1784,10 @@
         <v>45756</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D41" s="3">
         <v>40000</v>
@@ -1729,10 +1807,10 @@
         <v>45756</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D42" s="3">
         <v>14547</v>
@@ -1744,7 +1822,7 @@
         <v>3</v>
       </c>
       <c r="G42" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="43" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1752,10 +1830,10 @@
         <v>45756</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D43" s="3">
         <v>41500</v>
@@ -1767,7 +1845,7 @@
         <v>20</v>
       </c>
       <c r="G43" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="44" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1775,22 +1853,22 @@
         <v>45756</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D44" s="3">
         <v>41757</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="45" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1798,29 +1876,33 @@
         <v>45756</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D45" s="3">
         <v>40000</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="F45" s="4"/>
-      <c r="G45" s="4"/>
+        <v>51</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="G45" s="4" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="46" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="8">
         <v>45757</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D46" s="3">
         <v>14546</v>
@@ -1832,7 +1914,7 @@
         <v>3</v>
       </c>
       <c r="G46" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="47" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1840,16 +1922,16 @@
         <v>45757</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D47" s="3">
         <v>12611</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F47" s="4" t="s">
         <v>17</v>
@@ -1863,22 +1945,22 @@
         <v>45757</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D48" s="3">
         <v>16365</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G48" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="49" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -1886,48 +1968,56 @@
         <v>45757</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D49" s="3">
         <v>40000</v>
       </c>
       <c r="E49" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="F49" s="4"/>
-      <c r="G49" s="4"/>
+        <v>46</v>
+      </c>
+      <c r="F49" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="G49" s="4" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="50" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="8">
         <v>45757</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D50" s="3">
         <v>42900</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="F50" s="4"/>
-      <c r="G50" s="4"/>
+        <v>54</v>
+      </c>
+      <c r="F50" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G50" s="4" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="51" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="8">
         <v>45757</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D51" s="3">
         <v>40000</v>
@@ -1935,24 +2025,28 @@
       <c r="E51" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="F51" s="4"/>
-      <c r="G51" s="4"/>
+      <c r="F51" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="G51" s="4" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="52" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="8">
         <v>45758</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D52" s="3">
         <v>12728</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F52" s="4" t="s">
         <v>17</v>
@@ -1966,10 +2060,10 @@
         <v>45758</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D53" s="3">
         <v>14547</v>
@@ -1989,10 +2083,10 @@
         <v>45758</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C54" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D54" s="3">
         <v>14546</v>
@@ -2004,7 +2098,7 @@
         <v>3</v>
       </c>
       <c r="G54" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="55" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2012,10 +2106,10 @@
         <v>45758</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D55" s="3">
         <v>40000</v>
@@ -2023,30 +2117,34 @@
       <c r="E55" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F55" s="4"/>
-      <c r="G55" s="4"/>
+      <c r="F55" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="G55" s="4" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="56" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="8">
         <v>45758</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D56" s="3">
         <v>40000</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G56" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="57" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2054,10 +2152,10 @@
         <v>45758</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D57" s="3">
         <v>42277</v>
@@ -2066,10 +2164,10 @@
         <v>5</v>
       </c>
       <c r="F57" s="4" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G57" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="58" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2077,10 +2175,10 @@
         <v>45759</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D58" s="3">
         <v>36366</v>
@@ -2089,10 +2187,10 @@
         <v>5</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G58" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="59" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2100,16 +2198,16 @@
         <v>45760</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D59" s="3">
         <v>42725</v>
       </c>
       <c r="E59" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F59" s="4" t="s">
         <v>21</v>
@@ -2123,16 +2221,16 @@
         <v>45759</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D60" s="3">
         <v>14547</v>
       </c>
       <c r="E60" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F60" s="4" t="s">
         <v>15</v>
@@ -2146,10 +2244,10 @@
         <v>45759</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C61" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D61" s="3">
         <v>14000</v>
@@ -2161,7 +2259,7 @@
         <v>3</v>
       </c>
       <c r="G61" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="62" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2169,22 +2267,22 @@
         <v>45760</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C62" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D62" s="3">
         <v>14547</v>
       </c>
       <c r="E62" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F62" s="4" t="s">
         <v>3</v>
       </c>
       <c r="G62" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="63" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2192,16 +2290,16 @@
         <v>45760</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C63" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D63" s="3">
         <v>12728</v>
       </c>
       <c r="E63" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F63" s="4" t="s">
         <v>17</v>
@@ -2215,22 +2313,22 @@
         <v>45761</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D64" s="3">
         <v>41756</v>
       </c>
       <c r="E64" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G64" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="65" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2238,29 +2336,33 @@
         <v>45760</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D65" s="3">
         <v>43000</v>
       </c>
       <c r="E65" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="F65" s="4"/>
-      <c r="G65" s="4"/>
+        <v>55</v>
+      </c>
+      <c r="F65" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G65" s="4" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="66" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="8">
         <v>45760</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D66" s="3">
         <v>40000</v>
@@ -2268,37 +2370,45 @@
       <c r="E66" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="F66" s="4"/>
-      <c r="G66" s="4"/>
+      <c r="F66" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="G66" s="4" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="67" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="8">
         <v>45761</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D67" s="3">
         <v>40000</v>
       </c>
       <c r="E67" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="F67" s="4"/>
-      <c r="G67" s="4"/>
+        <v>54</v>
+      </c>
+      <c r="F67" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="G67" s="4" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="68" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="8">
         <v>45761</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D68" s="3">
         <v>12728</v>
@@ -2318,16 +2428,16 @@
         <v>45762</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D69" s="3">
         <v>14008</v>
       </c>
       <c r="E69" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F69" s="4" t="s">
         <v>15</v>
@@ -2341,29 +2451,33 @@
         <v>45762</v>
       </c>
       <c r="B70" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C70" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D70" s="3">
         <v>39830</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>47</v>
-      </c>
-      <c r="F70" s="4"/>
-      <c r="G70" s="4"/>
+        <v>46</v>
+      </c>
+      <c r="F70" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="G70" s="4" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="71" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="8">
         <v>45762</v>
       </c>
       <c r="B71" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C71" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D71" s="3">
         <v>43000</v>
@@ -2371,37 +2485,45 @@
       <c r="E71" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F71" s="4"/>
-      <c r="G71" s="4"/>
+      <c r="F71" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G71" s="4" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="72" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="8">
         <v>45762</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C72" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D72" s="3">
         <v>40000</v>
       </c>
       <c r="E72" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="F72" s="4"/>
-      <c r="G72" s="4"/>
+        <v>54</v>
+      </c>
+      <c r="F72" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="G72" s="4" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="73" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="8">
         <v>45764</v>
       </c>
       <c r="B73" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C73" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D73" s="3">
         <v>40000</v>
@@ -2421,10 +2543,10 @@
         <v>45764</v>
       </c>
       <c r="B74" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C74" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D74" s="3">
         <v>40000</v>
@@ -2436,7 +2558,7 @@
         <v>20</v>
       </c>
       <c r="G74" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="75" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2444,10 +2566,10 @@
         <v>45763</v>
       </c>
       <c r="B75" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C75" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D75" s="3">
         <v>40000</v>
@@ -2459,7 +2581,7 @@
         <v>2</v>
       </c>
       <c r="G75" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="76" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2467,22 +2589,22 @@
         <v>45764</v>
       </c>
       <c r="B76" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C76" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D76" s="3">
         <v>36368</v>
       </c>
       <c r="E76" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F76" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G76" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="77" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2490,22 +2612,22 @@
         <v>45764</v>
       </c>
       <c r="B77" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C77" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D77" s="3">
         <v>40457</v>
       </c>
       <c r="E77" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F77" s="4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G77" s="4" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="78" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2513,16 +2635,16 @@
         <v>45763</v>
       </c>
       <c r="B78" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C78" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D78" s="3">
         <v>14008</v>
       </c>
       <c r="E78" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F78" s="4" t="s">
         <v>15</v>
@@ -2536,22 +2658,22 @@
         <v>45764</v>
       </c>
       <c r="B79" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C79" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D79" s="3">
         <v>16365</v>
       </c>
       <c r="E79" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F79" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G79" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="80" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2559,29 +2681,33 @@
         <v>45765</v>
       </c>
       <c r="B80" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C80" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D80" s="3">
         <v>43000</v>
       </c>
       <c r="E80" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="F80" s="4"/>
-      <c r="G80" s="4"/>
+        <v>54</v>
+      </c>
+      <c r="F80" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G80" s="4" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="81" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="8">
         <v>45765</v>
       </c>
       <c r="B81" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D81" s="3">
         <v>14000</v>
@@ -2593,7 +2719,7 @@
         <v>3</v>
       </c>
       <c r="G81" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="82" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2601,10 +2727,10 @@
         <v>45765</v>
       </c>
       <c r="B82" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C82" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D82" s="3">
         <v>11070</v>
@@ -2624,16 +2750,16 @@
         <v>45765</v>
       </c>
       <c r="B83" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C83" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D83" s="3">
         <v>14547</v>
       </c>
       <c r="E83" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F83" s="4" t="s">
         <v>15</v>
@@ -2647,10 +2773,10 @@
         <v>45766</v>
       </c>
       <c r="B84" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C84" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D84" s="3">
         <v>12728</v>
@@ -2670,22 +2796,22 @@
         <v>45766</v>
       </c>
       <c r="B85" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C85" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D85" s="3">
         <v>14543</v>
       </c>
       <c r="E85" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F85" s="4" t="s">
         <v>3</v>
       </c>
       <c r="G85" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="86" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2693,22 +2819,22 @@
         <v>45766</v>
       </c>
       <c r="B86" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C86" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D86" s="3">
         <v>16362</v>
       </c>
       <c r="E86" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F86" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G86" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="87" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2716,16 +2842,16 @@
         <v>45767</v>
       </c>
       <c r="B87" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C87" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D87" s="3">
         <v>42725</v>
       </c>
       <c r="E87" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F87" s="4" t="s">
         <v>21</v>
@@ -2739,16 +2865,16 @@
         <v>45767</v>
       </c>
       <c r="B88" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C88" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D88" s="3">
         <v>13999</v>
       </c>
       <c r="E88" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F88" s="4" t="s">
         <v>15</v>
@@ -2762,10 +2888,10 @@
         <v>45767</v>
       </c>
       <c r="B89" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C89" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D89" s="3">
         <v>12187</v>
@@ -2785,10 +2911,10 @@
         <v>45767</v>
       </c>
       <c r="B90" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C90" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D90" s="3">
         <v>40000</v>
@@ -2796,87 +2922,103 @@
       <c r="E90" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F90" s="4"/>
-      <c r="G90" s="4"/>
+      <c r="F90" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="G90" s="4" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="91" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="8">
         <v>45767</v>
       </c>
       <c r="B91" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C91" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D91" s="3">
         <v>39900</v>
       </c>
       <c r="E91" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="F91" s="4"/>
-      <c r="G91" s="4"/>
+        <v>40</v>
+      </c>
+      <c r="F91" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="G91" s="4" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="92" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="8">
         <v>45767</v>
       </c>
       <c r="B92" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C92" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D92" s="3">
         <v>42730</v>
       </c>
       <c r="E92" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="F92" s="4"/>
-      <c r="G92" s="4"/>
+        <v>55</v>
+      </c>
+      <c r="F92" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G92" s="4" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="93" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="8">
         <v>45767</v>
       </c>
       <c r="B93" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C93" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D93" s="3">
         <v>40000</v>
       </c>
       <c r="E93" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="F93" s="4"/>
-      <c r="G93" s="4"/>
+        <v>51</v>
+      </c>
+      <c r="F93" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="G93" s="4" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="94" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="8">
         <v>45767</v>
       </c>
       <c r="B94" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C94" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D94" s="3">
         <v>13049</v>
       </c>
       <c r="E94" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F94" s="4" t="s">
         <v>3</v>
       </c>
       <c r="G94" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="95" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2884,10 +3026,10 @@
         <v>45768</v>
       </c>
       <c r="B95" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C95" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D95" s="3">
         <v>40010</v>
@@ -2896,10 +3038,10 @@
         <v>5</v>
       </c>
       <c r="F95" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G95" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="96" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2907,16 +3049,16 @@
         <v>45768</v>
       </c>
       <c r="B96" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C96" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D96" s="3">
         <v>12728</v>
       </c>
       <c r="E96" s="6" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F96" s="4" t="s">
         <v>17</v>
@@ -2930,22 +3072,22 @@
         <v>45768</v>
       </c>
       <c r="B97" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D97" s="3">
         <v>16102</v>
       </c>
       <c r="E97" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F97" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G97" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="98" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -2953,35 +3095,39 @@
         <v>45769</v>
       </c>
       <c r="B98" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C98" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D98" s="3">
         <v>42612</v>
       </c>
       <c r="E98" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="F98" s="4"/>
-      <c r="G98" s="4"/>
+        <v>54</v>
+      </c>
+      <c r="F98" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G98" s="4" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="99" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="8">
         <v>45769</v>
       </c>
       <c r="B99" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C99" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D99" s="3">
         <v>14342</v>
       </c>
       <c r="E99" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F99" s="4" t="s">
         <v>15</v>
@@ -2995,10 +3141,10 @@
         <v>45769</v>
       </c>
       <c r="B100" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C100" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D100" s="3">
         <v>40000</v>
@@ -3007,10 +3153,10 @@
         <v>5</v>
       </c>
       <c r="F100" s="4" t="s">
-        <v>22</v>
+        <v>88</v>
       </c>
       <c r="G100" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="101" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -3018,10 +3164,10 @@
         <v>45769</v>
       </c>
       <c r="B101" s="6" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C101" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D101" s="3">
         <v>40000</v>
@@ -3029,18 +3175,22 @@
       <c r="E101" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F101" s="4"/>
-      <c r="G101" s="4"/>
+      <c r="F101" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="G101" s="4" t="s">
+        <v>83</v>
+      </c>
     </row>
     <row r="102" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="8">
         <v>45770</v>
       </c>
       <c r="B102" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C102" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D102" s="3">
         <v>41500</v>
@@ -3060,16 +3210,16 @@
         <v>45770</v>
       </c>
       <c r="B103" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C103" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D103" s="3">
         <v>12728</v>
       </c>
       <c r="E103" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F103" s="4" t="s">
         <v>17</v>
@@ -3083,22 +3233,22 @@
         <v>45771</v>
       </c>
       <c r="B104" s="6" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="C104" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D104" s="3">
         <v>41757</v>
       </c>
       <c r="E104" s="6" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F104" s="4" t="s">
         <v>1</v>
       </c>
       <c r="G104" s="4" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
     </row>
     <row r="105" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -3106,22 +3256,22 @@
         <v>45771</v>
       </c>
       <c r="B105" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C105" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D105" s="3">
         <v>16365</v>
       </c>
       <c r="E105" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F105" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G105" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="106" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -3129,10 +3279,10 @@
         <v>45771</v>
       </c>
       <c r="B106" s="6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C106" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D106" s="3">
         <v>42277</v>
@@ -3144,7 +3294,7 @@
         <v>16</v>
       </c>
       <c r="G106" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="107" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -3152,10 +3302,10 @@
         <v>45772</v>
       </c>
       <c r="B107" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C107" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D107" s="3">
         <v>40000</v>
@@ -3163,49 +3313,57 @@
       <c r="E107" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F107" s="4"/>
-      <c r="G107" s="4"/>
+      <c r="F107" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="G107" s="4" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="108" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="8">
         <v>45772</v>
       </c>
       <c r="B108" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C108" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D108" s="3">
         <v>40000</v>
       </c>
       <c r="E108" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="F108" s="4"/>
-      <c r="G108" s="4"/>
+        <v>54</v>
+      </c>
+      <c r="F108" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="G108" s="4" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="109" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="8">
         <v>45772</v>
       </c>
       <c r="B109" s="6" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="C109" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D109" s="3">
         <v>36368</v>
       </c>
       <c r="E109" s="6" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F109" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="G109" s="4" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="110" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -3213,10 +3371,10 @@
         <v>45772</v>
       </c>
       <c r="B110" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C110" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D110" s="3">
         <v>14546</v>
@@ -3228,7 +3386,7 @@
         <v>3</v>
       </c>
       <c r="G110" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="111" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -3236,16 +3394,16 @@
         <v>45772</v>
       </c>
       <c r="B111" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C111" s="2" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D111" s="3">
         <v>12728</v>
       </c>
       <c r="E111" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F111" s="4" t="s">
         <v>17</v>
@@ -3259,29 +3417,33 @@
         <v>45772</v>
       </c>
       <c r="B112" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C112" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D112" s="3">
         <v>40000</v>
       </c>
       <c r="E112" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="F112" s="4"/>
-      <c r="G112" s="4"/>
+        <v>54</v>
+      </c>
+      <c r="F112" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="G112" s="4" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="113" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A113" s="8">
         <v>45773</v>
       </c>
       <c r="B113" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C113" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D113" s="3">
         <v>14547</v>
@@ -3293,7 +3455,7 @@
         <v>3</v>
       </c>
       <c r="G113" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="114" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -3301,16 +3463,16 @@
         <v>45773</v>
       </c>
       <c r="B114" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C114" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D114" s="3">
         <v>14547</v>
       </c>
       <c r="E114" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F114" s="4" t="s">
         <v>15</v>
@@ -3324,10 +3486,10 @@
         <v>45773</v>
       </c>
       <c r="B115" s="6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="C115" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D115" s="3">
         <v>43000</v>
@@ -3335,30 +3497,34 @@
       <c r="E115" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="F115" s="4"/>
-      <c r="G115" s="4"/>
+      <c r="F115" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="G115" s="4" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="116" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A116" s="8">
         <v>45773</v>
       </c>
       <c r="B116" s="6" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C116" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D116" s="3">
         <v>16365</v>
       </c>
       <c r="E116" s="6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F116" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="G116" s="4" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="117" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -3366,16 +3532,16 @@
         <v>45773</v>
       </c>
       <c r="B117" s="6" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C117" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D117" s="3">
         <v>42725</v>
       </c>
       <c r="E117" s="6" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F117" s="4" t="s">
         <v>21</v>
@@ -3389,10 +3555,10 @@
         <v>45774</v>
       </c>
       <c r="B118" s="6" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C118" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D118" s="3">
         <v>14540</v>
@@ -3404,7 +3570,7 @@
         <v>3</v>
       </c>
       <c r="G118" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
     </row>
     <row r="119" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -3412,29 +3578,33 @@
         <v>45774</v>
       </c>
       <c r="B119" s="6" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C119" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D119" s="3">
         <v>43000</v>
       </c>
       <c r="E119" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="F119" s="4"/>
-      <c r="G119" s="4"/>
+        <v>40</v>
+      </c>
+      <c r="F119" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="G119" s="4" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="120" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A120" s="8">
         <v>45774</v>
       </c>
       <c r="B120" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C120" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D120" s="3">
         <v>12728</v>
@@ -3454,16 +3624,16 @@
         <v>45774</v>
       </c>
       <c r="B121" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C121" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D121" s="3">
         <v>14547</v>
       </c>
       <c r="E121" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F121" s="4" t="s">
         <v>15</v>
@@ -3477,10 +3647,10 @@
         <v>45774</v>
       </c>
       <c r="B122" s="6" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C122" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D122" s="3">
         <v>40004</v>
@@ -3500,22 +3670,22 @@
         <v>45775</v>
       </c>
       <c r="B123" s="6" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C123" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D123" s="3">
         <v>39140</v>
       </c>
       <c r="E123" s="6" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F123" s="4" t="s">
-        <v>22</v>
+        <v>88</v>
       </c>
       <c r="G123" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="124" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -3523,10 +3693,10 @@
         <v>45776</v>
       </c>
       <c r="B124" s="6" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C124" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D124" s="3">
         <v>39500</v>
@@ -3538,7 +3708,7 @@
         <v>2</v>
       </c>
       <c r="G124" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="125" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -3546,10 +3716,10 @@
         <v>45776</v>
       </c>
       <c r="B125" s="6" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C125" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D125" s="3">
         <v>40000</v>
@@ -3558,10 +3728,10 @@
         <v>5</v>
       </c>
       <c r="F125" s="4" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G125" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="126" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -3569,10 +3739,10 @@
         <v>45776</v>
       </c>
       <c r="B126" s="6" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C126" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D126" s="3">
         <v>41500</v>
@@ -3584,7 +3754,7 @@
         <v>20</v>
       </c>
       <c r="G126" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
     </row>
     <row r="127" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -3592,10 +3762,10 @@
         <v>45776</v>
       </c>
       <c r="B127" s="6" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C127" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D127" s="3">
         <v>40000</v>
@@ -3603,43 +3773,51 @@
       <c r="E127" s="6" t="s">
         <v>6</v>
       </c>
-      <c r="F127" s="4"/>
-      <c r="G127" s="4"/>
+      <c r="F127" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="G127" s="4" t="s">
+        <v>81</v>
+      </c>
     </row>
     <row r="128" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A128" s="8">
         <v>45776</v>
       </c>
       <c r="B128" s="6" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C128" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D128" s="3">
         <v>40000</v>
       </c>
       <c r="E128" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="F128" s="4"/>
-      <c r="G128" s="4"/>
+        <v>54</v>
+      </c>
+      <c r="F128" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="G128" s="4" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="129" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A129" s="8">
         <v>45776</v>
       </c>
       <c r="B129" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C129" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D129" s="3">
         <v>14547</v>
       </c>
       <c r="E129" s="6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F129" s="4" t="s">
         <v>15</v>
@@ -3653,35 +3831,39 @@
         <v>45777</v>
       </c>
       <c r="B130" s="6" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="C130" s="6" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D130" s="3">
         <v>40000</v>
       </c>
       <c r="E130" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="F130" s="4"/>
-      <c r="G130" s="4"/>
+        <v>54</v>
+      </c>
+      <c r="F130" s="4" t="s">
+        <v>84</v>
+      </c>
+      <c r="G130" s="4" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="131" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A131" s="8">
         <v>45777</v>
       </c>
       <c r="B131" s="6" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C131" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D131" s="3">
         <v>14539</v>
       </c>
       <c r="E131" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F131" s="4" t="s">
         <v>15</v>
@@ -3695,16 +3877,16 @@
         <v>45777</v>
       </c>
       <c r="B132" s="6" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C132" s="6" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D132" s="3">
         <v>12728</v>
       </c>
       <c r="E132" s="6" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F132" s="4" t="s">
         <v>17</v>
@@ -3715,14 +3897,6 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:G132" xr:uid="{3DD6E5EE-1A2B-42A0-908A-454201FDD3D7}"/>
-  <dataValidations count="2">
-    <dataValidation type="list" errorStyle="warning" allowBlank="1" showErrorMessage="1" errorTitle="Typing Issue" error="Pls, type your text correctly." sqref="B2:C131" xr:uid="{991CF2B9-B32D-4651-9E33-2F34AC34FC8C}">
-      <formula1>#REF!</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C105 C103 C30 C99 C10 C94 C12 C42 C110:C111 C96:C97 C88:C89 C81:C86 C78:C79 C68:C69 C60:C63 C52:C54 C46:C48 C37:C39 C32:C34 C23:C24 C15:C19 C2:C4 F2:G132" xr:uid="{F5E42C72-12A3-4CB7-8C15-86FC57CBA65E}">
-      <formula1>#REF!</formula1>
-    </dataValidation>
-  </dataValidations>
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.2" right="0.2" top="0.2" bottom="0.2" header="0" footer="0"/>
   <pageSetup paperSize="9" scale="10" fitToHeight="0" orientation="landscape" horizontalDpi="4294967293" r:id="rId1"/>

</xml_diff>